<commit_message>
mise à jour du portfolio
</commit_message>
<xml_diff>
--- a/8-1 - BTS SIO - 2025 - Annexe 8-1 - Epreuve E5 - Tableau de synthese.xlsx
+++ b/8-1 - BTS SIO - 2025 - Annexe 8-1 - Epreuve E5 - Tableau de synthese.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29910"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\BTS\2025\CIRCULAIRES NATIONALES\SIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E42AB7D6-9DA0-B145-815D-5CEF1CC99B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="8_{E42AB7D6-9DA0-B145-815D-5CEF1CC99B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC65E7AD-FE78-48B0-84E7-1D97F557BFD9}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,6 +20,9 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -36,7 +39,45 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+  <si>
+    <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
+  </si>
+  <si>
+    <t>SESSION 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tableau de synthèse des réalisations professionnelles </t>
+  </si>
+  <si>
+    <t>NOM et prénom : OTHMAN Soraya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N° candidat : </t>
+  </si>
+  <si>
+    <t>Centre de formation : H3 Hitema</t>
+  </si>
+  <si>
+    <t>Option :</t>
+  </si>
+  <si>
+    <t>▢ SISR</t>
+  </si>
+  <si>
+    <t>▢ SLAM</t>
+  </si>
+  <si>
+    <t>Adresse URL du portfolio :</t>
+  </si>
+  <si>
+    <t>Compétences mises en œuvre
+Réalisations professionnelles
+(intitulé et liste des documents et productions associés)</t>
+  </si>
+  <si>
+    <t>Période (sous la forme du JJ/MM/AA au JJ/MM/AA)</t>
+  </si>
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -54,15 +95,6 @@
   </si>
   <si>
     <t>Organiser son développement professionnel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tableau de synthèse des réalisations professionnelles </t>
-  </si>
-  <si>
-    <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
-  </si>
-  <si>
-    <t>Option :</t>
   </si>
   <si>
     <t>▸Recenser et identifier les ressources numériques 
@@ -99,53 +131,61 @@
 ▸Développer son projet professionnel</t>
   </si>
   <si>
-    <t>Centre de formation :</t>
-  </si>
-  <si>
-    <t>▢ SISR</t>
-  </si>
-  <si>
-    <t>▢ SLAM</t>
-  </si>
-  <si>
     <t xml:space="preserve">Réalisation en cours de formation
 </t>
   </si>
   <si>
-    <t>Compétences mises en œuvre
-Réalisations professionnelles
-(intitulé et liste des documents et productions associés)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N° candidat : </t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOM et prénom : </t>
-  </si>
-  <si>
-    <t>Période (sous la forme du JJ/MM/AA au JJ/MM/AA)</t>
+    <t>Exercice Openclassroom, création d'un portefolio pour une photographe
+HTML,CSS</t>
+  </si>
+  <si>
+    <t>Création d'un site E-commerce « Fiestita »
+HTML,CSS</t>
+  </si>
+  <si>
+    <t>Création d'un site E-commerce pour des locations de voiture
+HTML,CSS,SQL,PHP</t>
+  </si>
+  <si>
+    <t>Exercice création d'un « Tétris »
+HTML,CSS,Javascript</t>
+  </si>
+  <si>
+    <t>Création d'une application de billeterie Java,SQL,JavaFX</t>
+  </si>
+  <si>
+    <t>Création d'une application Web d'un bibliothèque en ligne Php,Laravel,HTML,CSS,Javascript</t>
   </si>
   <si>
     <t>Réalisations en milieu professionnel en cours de première année</t>
   </si>
   <si>
+    <t>Développement  d'une application de gestion de stock durant un stage dans l'entreprise « Sonis »
+HTML,CSS,Node,js,SQL,Javascript</t>
+  </si>
+  <si>
+    <t>31/03/2025
+15/05/2025</t>
+  </si>
+  <si>
     <t>Réalisations en milieu professionnel en cours de seconde année</t>
   </si>
   <si>
-    <t>Adresse URL du portfolio :</t>
-  </si>
-  <si>
-    <t>SESSION 2025</t>
+    <t>Modification,ajout et correction d'une application de gestion de stock durant un stage dans l'entreprise "Sonis" et nettoyage de la bases de données "Client" (Suppression des doublons, correction des mauvaisse saisies, vérifier les valeurs si elles sont encore valides, ajout de valeurs manquante) de l'entreprise. SQL</t>
+  </si>
+  <si>
+    <t>15/12/2025 au 31/01/2025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -203,20 +243,43 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <sz val="16"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF70AD47"/>
+        <bgColor rgb="FF70AD47"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="29">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -602,12 +665,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF4A452A"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF4A452A"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF4A452A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF4A452A"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -615,9 +693,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -630,18 +705,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -651,18 +714,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -684,9 +741,42 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -711,44 +801,57 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -766,6 +869,107 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>390525</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="2" name="">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8EED6288-4C80-4881-A291-400F400BA28B}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="11877675" y="1619250"/>
+            <a:ext cx="161925" cy="276225"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="2" name="">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8EED6288-4C80-4881-A291-400F400BA28B}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="11859358" y="1601718"/>
+              <a:ext cx="198193" cy="311648"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/ink/ink1.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+          <inkml:channel name="OA" type="integer" max="360" units="deg"/>
+          <inkml:channel name="OE" type="integer" max="90" units="deg"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+          <inkml:channelProperty channel="OA" name="resolution" value="1000" units="1/deg"/>
+          <inkml:channelProperty channel="OE" name="resolution" value="1000" units="1/deg"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.1" units="cm"/>
+      <inkml:brushProperty name="height" value="0.1" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">25977 4498 16383 0 0,'0'4'0'0'0,"0"7"0"0"0,0 14 0 0 0,0 10 0 0 0,0 5 0 0 0,0 4 0 0 0,0 5 0 0 0,0-3 0 0 0,0-4 0 0 0,0-7 0 0 0,0-6 0 0 0,0-3 0 0 0,0-3 0 0 0,0-2 0 0 0,3-5 0 0 0,6-1 0 0 0,4-3 0 0 0,0 0 0 0 0,1-2 0 0 0,3 1 0 0 0,1-2 0 0 0,1 5 0 0 0,2 4 0 0 0,-4 2 0 0 0,-4 2 0 0 0,-1 0 0 0 0,-2 4 0 0 0,0 1 0 0 0,-1 0 0 0 0,2-6 0 0 0,-2-1 0 0 0,2-5 0 0 0,-2-2 0 0 0,-1-2 0 0 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="0.14">26337 4667 16383 0 0,'-4'0'0'0'0,"-4"0"0"0"0,-2 4 0 0 0,-2 1 0 0 0,-2 3 0 0 0,0 4 0 0 0,3 3 0 0 0,4 4 0 0 0,-1-3 0 0 0,1 1 0 0 0,-2-4 0 0 0,0 1 0 0 0,-1-3 0 0 0,0 0 0 0 0,-1 3 0 0 0,1 5 0 0 0,-1 0 0 0 0,1 0 0 0 0,-1 1 0 0 0,1 0 0 0 0,2 1 0 0 0,-1-4 0 0 0,-2-1 0 0 0,0 1 0 0 0,2 0 0 0 0,-1-2 0 0 0,2 0 0 0 0,-2-3 0 0 0,0 1 0 0 0,0-3 0 0 0,-4-2 0 0 0,-2-3 0 0 0,-2-2 0 0 0,-1-2 0 0 0,-2-1 0 0 0,-1 0 0 0 0,4 3 0 0 0,5 5 0 0 0,4 1 0 0 0</inkml:trace>
+</inkml:ink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1059,134 +1263,134 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AQ81"/>
-  <sheetFormatPr defaultColWidth="10.78515625" defaultRowHeight="12.75" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="70.390625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.78515625" style="1" customWidth="1"/>
-    <col min="3" max="8" width="18.7421875" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.4609375" customWidth="1"/>
-    <col min="44" max="16384" width="10.78515625" style="1"/>
+    <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" style="51" customWidth="1"/>
+    <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
+    <col min="9" max="43" width="11.42578125" customWidth="1"/>
+    <col min="44" max="16384" width="10.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="26"/>
-    </row>
-    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-    </row>
-    <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="27" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="33" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" s="28"/>
-      <c r="H3" s="34"/>
+    <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1">
+      <c r="A1" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="21"/>
+    </row>
+    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1">
+      <c r="A2" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+    </row>
+    <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1">
+      <c r="A3" s="31" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="37" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="32"/>
+      <c r="H3" s="38"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="30" t="s">
+    <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1">
+      <c r="A4" s="34" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1">
+      <c r="A5" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="30"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1">
+      <c r="A6" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="44" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="17" t="s">
+      <c r="G6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="H6" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="45" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="46"/>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
-      <c r="F5" s="46"/>
-      <c r="G5" s="46"/>
-      <c r="H5" s="47"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="35" t="s">
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1">
+      <c r="A7" s="20"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="55" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="43" t="s">
+      <c r="E7" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="36"/>
-      <c r="B7" s="44"/>
-      <c r="C7" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>14</v>
+      <c r="H7" s="56" t="s">
+        <v>23</v>
       </c>
       <c r="I7"/>
       <c r="J7"/>
@@ -1224,17 +1428,17 @@
       <c r="AP7"/>
       <c r="AQ7"/>
     </row>
-    <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.15">
-      <c r="A8" s="37" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="38"/>
-      <c r="C8" s="38"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="38"/>
-      <c r="G8" s="38"/>
-      <c r="H8" s="39"/>
+    <row r="8" spans="1:43" s="2" customFormat="1" ht="18">
+      <c r="A8" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="24"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1271,15 +1475,19 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="12"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="20"/>
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A9" s="52" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="39">
+        <v>45444</v>
+      </c>
+      <c r="C9" s="40"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="41"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="41"/>
+      <c r="H9" s="42"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1316,15 +1524,19 @@
       <c r="AP9"/>
       <c r="AQ9"/>
     </row>
-    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="12"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="20"/>
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A10" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="39">
+        <v>45536</v>
+      </c>
+      <c r="C10" s="43"/>
+      <c r="D10" s="43"/>
+      <c r="E10" s="43"/>
+      <c r="F10" s="42"/>
+      <c r="G10" s="43"/>
+      <c r="H10" s="41"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1361,15 +1573,19 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="12"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="20"/>
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A11" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="39">
+        <v>45611</v>
+      </c>
+      <c r="C11" s="43"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="43"/>
+      <c r="H11" s="41"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1406,15 +1622,19 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="12"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="20"/>
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A12" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="39">
+        <v>45726</v>
+      </c>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="13"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1451,15 +1671,19 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="12"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="20"/>
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A13" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="39">
+        <v>45931</v>
+      </c>
+      <c r="C13" s="43"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="42"/>
+      <c r="F13" s="42"/>
+      <c r="G13" s="43"/>
+      <c r="H13" s="43"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1496,15 +1720,19 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="12"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="20"/>
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A14" s="52" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="39">
+        <v>46082</v>
+      </c>
+      <c r="C14" s="43"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="42"/>
+      <c r="H14" s="43"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1541,15 +1769,15 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="12"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="20"/>
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A15" s="52"/>
+      <c r="B15" s="39"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="13"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1586,15 +1814,15 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="12"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="20"/>
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A16" s="7"/>
+      <c r="B16" s="46"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="13"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1631,15 +1859,15 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="12"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="20"/>
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A17" s="7"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="13"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1676,15 +1904,15 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="12"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="20"/>
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A18" s="7"/>
+      <c r="B18" s="46"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="13"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1721,17 +1949,17 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.15">
-      <c r="A19" s="40" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="41"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="41"/>
-      <c r="E19" s="41"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="41"/>
-      <c r="H19" s="42"/>
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="18">
+      <c r="A19" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="27"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1768,15 +1996,19 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="12"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="20"/>
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A20" s="52" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" s="53" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="42"/>
+      <c r="D20" s="42"/>
+      <c r="E20" s="42"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="42"/>
+      <c r="H20" s="43"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1813,15 +2045,15 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="12"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="20"/>
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A21" s="7"/>
+      <c r="B21" s="46"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="13"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1858,15 +2090,15 @@
       <c r="AP21"/>
       <c r="AQ21"/>
     </row>
-    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="12"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="20"/>
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A22" s="7"/>
+      <c r="B22" s="46"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="13"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -1903,15 +2135,15 @@
       <c r="AP22"/>
       <c r="AQ22"/>
     </row>
-    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="12"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="20"/>
+    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A23" s="7"/>
+      <c r="B23" s="46"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="13"/>
       <c r="I23"/>
       <c r="J23"/>
       <c r="K23"/>
@@ -1948,15 +2180,15 @@
       <c r="AP23"/>
       <c r="AQ23"/>
     </row>
-    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="12"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="20"/>
+    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A24" s="7"/>
+      <c r="B24" s="46"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="13"/>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -1993,15 +2225,15 @@
       <c r="AP24"/>
       <c r="AQ24"/>
     </row>
-    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A25" s="12"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="20"/>
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A25" s="7"/>
+      <c r="B25" s="46"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="13"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -2038,15 +2270,15 @@
       <c r="AP25"/>
       <c r="AQ25"/>
     </row>
-    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="12"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="20"/>
+    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A26" s="7"/>
+      <c r="B26" s="46"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="13"/>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2083,17 +2315,17 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.15">
-      <c r="A27" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="B27" s="41"/>
-      <c r="C27" s="41"/>
-      <c r="D27" s="41"/>
-      <c r="E27" s="41"/>
-      <c r="F27" s="41"/>
-      <c r="G27" s="41"/>
-      <c r="H27" s="42"/>
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="18">
+      <c r="A27" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="26"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="27"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2130,15 +2362,19 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A28" s="12"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="20"/>
+    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A28" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" s="54" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" s="42"/>
+      <c r="D28" s="42"/>
+      <c r="E28" s="42"/>
+      <c r="F28" s="42"/>
+      <c r="G28" s="42"/>
+      <c r="H28" s="43"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2175,15 +2411,15 @@
       <c r="AP28"/>
       <c r="AQ28"/>
     </row>
-    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="12"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="19"/>
-      <c r="H29" s="20"/>
+    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A29" s="7"/>
+      <c r="B29" s="46"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="13"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2220,15 +2456,15 @@
       <c r="AP29"/>
       <c r="AQ29"/>
     </row>
-    <row r="30" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="12"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="20"/>
+    <row r="30" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A30" s="7"/>
+      <c r="B30" s="46"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="13"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2265,15 +2501,15 @@
       <c r="AP30"/>
       <c r="AQ30"/>
     </row>
-    <row r="31" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A31" s="12"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="20"/>
+    <row r="31" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A31" s="7"/>
+      <c r="B31" s="46"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="13"/>
       <c r="I31"/>
       <c r="J31"/>
       <c r="K31"/>
@@ -2310,15 +2546,15 @@
       <c r="AP31"/>
       <c r="AQ31"/>
     </row>
-    <row r="32" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A32" s="12"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="19"/>
-      <c r="H32" s="20"/>
+    <row r="32" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A32" s="7"/>
+      <c r="B32" s="46"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="12"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="13"/>
       <c r="I32"/>
       <c r="J32"/>
       <c r="K32"/>
@@ -2355,15 +2591,15 @@
       <c r="AP32"/>
       <c r="AQ32"/>
     </row>
-    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A33" s="13"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="21"/>
-      <c r="F33" s="21"/>
-      <c r="G33" s="21"/>
-      <c r="H33" s="22"/>
+    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A33" s="8"/>
+      <c r="B33" s="47"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="15"/>
       <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
@@ -2400,15 +2636,15 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="14"/>
-      <c r="B34" s="15"/>
-      <c r="C34" s="23"/>
-      <c r="D34" s="23"/>
-      <c r="E34" s="23"/>
-      <c r="F34" s="23"/>
-      <c r="G34" s="23"/>
-      <c r="H34" s="24"/>
+    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1">
+      <c r="A34" s="9"/>
+      <c r="B34" s="48"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="16"/>
+      <c r="H34" s="17"/>
       <c r="I34"/>
       <c r="J34"/>
       <c r="K34"/>
@@ -2445,15 +2681,15 @@
       <c r="AP34"/>
       <c r="AQ34"/>
     </row>
-    <row r="35" spans="1:43" s="2" customFormat="1" ht="13.5" x14ac:dyDescent="0.15">
-      <c r="A35" s="5"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
+    <row r="35" spans="1:43" s="2" customFormat="1" ht="13.5">
+      <c r="A35" s="4"/>
+      <c r="B35" s="49"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
       <c r="I35"/>
       <c r="J35"/>
       <c r="K35"/>
@@ -2490,54 +2726,151 @@
       <c r="AP35"/>
       <c r="AQ35"/>
     </row>
-    <row r="36" spans="1:43" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="49" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="50" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="51" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="52" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="53" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="54" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="55" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="56" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="57" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="58" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="59" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="60" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="61" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="62" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="63" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="64" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="65" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="66" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="67" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="68" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="69" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="70" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="71" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="72" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="73" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="74" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="75" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="76" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="77" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="78" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="79" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="80" customFormat="1" x14ac:dyDescent="0.15"/>
-    <row r="81" customFormat="1" x14ac:dyDescent="0.15"/>
+    <row r="36" spans="1:43" customFormat="1">
+      <c r="B36" s="50"/>
+    </row>
+    <row r="37" spans="1:43" customFormat="1">
+      <c r="B37" s="50"/>
+    </row>
+    <row r="38" spans="1:43" customFormat="1">
+      <c r="B38" s="50"/>
+    </row>
+    <row r="39" spans="1:43" customFormat="1">
+      <c r="B39" s="50"/>
+    </row>
+    <row r="40" spans="1:43" customFormat="1">
+      <c r="B40" s="50"/>
+    </row>
+    <row r="41" spans="1:43" customFormat="1">
+      <c r="B41" s="50"/>
+    </row>
+    <row r="42" spans="1:43" customFormat="1">
+      <c r="B42" s="50"/>
+    </row>
+    <row r="43" spans="1:43" customFormat="1">
+      <c r="B43" s="50"/>
+    </row>
+    <row r="44" spans="1:43" customFormat="1">
+      <c r="B44" s="50"/>
+    </row>
+    <row r="45" spans="1:43" customFormat="1">
+      <c r="B45" s="50"/>
+    </row>
+    <row r="46" spans="1:43" customFormat="1">
+      <c r="B46" s="50"/>
+    </row>
+    <row r="47" spans="1:43" customFormat="1">
+      <c r="B47" s="50"/>
+    </row>
+    <row r="48" spans="1:43" customFormat="1">
+      <c r="B48" s="50"/>
+    </row>
+    <row r="49" spans="2:2" customFormat="1">
+      <c r="B49" s="50"/>
+    </row>
+    <row r="50" spans="2:2" customFormat="1">
+      <c r="B50" s="50"/>
+    </row>
+    <row r="51" spans="2:2" customFormat="1">
+      <c r="B51" s="50"/>
+    </row>
+    <row r="52" spans="2:2" customFormat="1">
+      <c r="B52" s="50"/>
+    </row>
+    <row r="53" spans="2:2" customFormat="1">
+      <c r="B53" s="50"/>
+    </row>
+    <row r="54" spans="2:2" customFormat="1">
+      <c r="B54" s="50"/>
+    </row>
+    <row r="55" spans="2:2" customFormat="1">
+      <c r="B55" s="50"/>
+    </row>
+    <row r="56" spans="2:2" customFormat="1">
+      <c r="B56" s="50"/>
+    </row>
+    <row r="57" spans="2:2" customFormat="1">
+      <c r="B57" s="50"/>
+    </row>
+    <row r="58" spans="2:2" customFormat="1">
+      <c r="B58" s="50"/>
+    </row>
+    <row r="59" spans="2:2" customFormat="1">
+      <c r="B59" s="50"/>
+    </row>
+    <row r="60" spans="2:2" customFormat="1">
+      <c r="B60" s="50"/>
+    </row>
+    <row r="61" spans="2:2" customFormat="1">
+      <c r="B61" s="50"/>
+    </row>
+    <row r="62" spans="2:2" customFormat="1">
+      <c r="B62" s="50"/>
+    </row>
+    <row r="63" spans="2:2" customFormat="1">
+      <c r="B63" s="50"/>
+    </row>
+    <row r="64" spans="2:2" customFormat="1">
+      <c r="B64" s="50"/>
+    </row>
+    <row r="65" spans="2:2" customFormat="1">
+      <c r="B65" s="50"/>
+    </row>
+    <row r="66" spans="2:2" customFormat="1">
+      <c r="B66" s="50"/>
+    </row>
+    <row r="67" spans="2:2" customFormat="1">
+      <c r="B67" s="50"/>
+    </row>
+    <row r="68" spans="2:2" customFormat="1">
+      <c r="B68" s="50"/>
+    </row>
+    <row r="69" spans="2:2" customFormat="1">
+      <c r="B69" s="50"/>
+    </row>
+    <row r="70" spans="2:2" customFormat="1">
+      <c r="B70" s="50"/>
+    </row>
+    <row r="71" spans="2:2" customFormat="1">
+      <c r="B71" s="50"/>
+    </row>
+    <row r="72" spans="2:2" customFormat="1">
+      <c r="B72" s="50"/>
+    </row>
+    <row r="73" spans="2:2" customFormat="1">
+      <c r="B73" s="50"/>
+    </row>
+    <row r="74" spans="2:2" customFormat="1">
+      <c r="B74" s="50"/>
+    </row>
+    <row r="75" spans="2:2" customFormat="1">
+      <c r="B75" s="50"/>
+    </row>
+    <row r="76" spans="2:2" customFormat="1">
+      <c r="B76" s="50"/>
+    </row>
+    <row r="77" spans="2:2" customFormat="1">
+      <c r="B77" s="50"/>
+    </row>
+    <row r="78" spans="2:2" customFormat="1">
+      <c r="B78" s="50"/>
+    </row>
+    <row r="79" spans="2:2" customFormat="1">
+      <c r="B79" s="50"/>
+    </row>
+    <row r="80" spans="2:2" customFormat="1">
+      <c r="B80" s="50"/>
+    </row>
+    <row r="81" spans="2:2" customFormat="1">
+      <c r="B81" s="50"/>
+    </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2545,16 +2878,12 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="48" orientation="portrait"/>
   <headerFooter alignWithMargins="0"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>